<commit_message>
chore: track project skills and lockfile, refresh machine workbook
Add the ProdPlan workflow skills (commit-and-push, feature-start,
feature-done) and package-lock.json so installs are reproducible.
Ignore the _to_delete/ scratch folder.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Machine/Machines.xlsx
+++ b/Machine/Machines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AI\ProdPlan\Machine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9296F6E-354A-4DDE-8B71-F6AE04734FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D282B98E-C061-4A37-96C6-F6C509EE68E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Furnace 1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="22">
   <si>
     <t>Name</t>
   </si>
@@ -456,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AM21"/>
+  <dimension ref="A1:AK21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" bestFit="1" customWidth="1"/>
@@ -519,7 +519,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="20" spans="1:39" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -537,7 +537,7 @@
         <v>3</v>
       </c>
       <c r="F20">
-        <f t="shared" ref="F20:AL20" si="0">E20+1</f>
+        <f t="shared" ref="F20:AJ20" si="0">E20+1</f>
         <v>4</v>
       </c>
       <c r="G20">
@@ -660,16 +660,8 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="AK20">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-      <c r="AL20">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" spans="1:39" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -744,10 +736,10 @@
       <c r="X21">
         <v>1000</v>
       </c>
-      <c r="AL21">
-        <v>200</v>
-      </c>
-      <c r="AM21" t="s">
+      <c r="AJ21">
+        <v>300</v>
+      </c>
+      <c r="AK21" t="s">
         <v>11</v>
       </c>
     </row>
@@ -758,7 +750,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36BE85E0-FB0B-42C3-B38A-F5ED44818443}">
-  <dimension ref="A1:AM21"/>
+  <dimension ref="A1:AK21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" bestFit="1" customWidth="1"/>
@@ -821,7 +813,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="20" spans="1:39" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -962,16 +954,8 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="AK20">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-      <c r="AL20">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" spans="1:39" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1046,10 +1030,10 @@
       <c r="X21">
         <v>1000</v>
       </c>
-      <c r="AL21">
-        <v>200</v>
-      </c>
-      <c r="AM21" t="s">
+      <c r="AJ21">
+        <v>300</v>
+      </c>
+      <c r="AK21" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1124,6 +1108,9 @@
       </c>
     </row>
     <row r="20" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
       <c r="B20">
         <v>0</v>
       </c>
@@ -1740,7 +1727,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6835B0CD-A8C8-4A7B-A7E9-86AAA5AF77E1}">
-  <dimension ref="A1:AM21"/>
+  <dimension ref="A1:AK21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" bestFit="1" customWidth="1"/>
@@ -1803,7 +1790,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="20" spans="1:39" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -1944,16 +1931,8 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="AK20">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-      <c r="AL20">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" spans="1:39" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -2028,10 +2007,10 @@
       <c r="X21">
         <v>1000</v>
       </c>
-      <c r="AL21">
-        <v>200</v>
-      </c>
-      <c r="AM21" t="s">
+      <c r="AJ21">
+        <v>300</v>
+      </c>
+      <c r="AK21" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2042,7 +2021,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC81CA44-2003-42C0-87B1-6F07DAD63A52}">
-  <dimension ref="A1:AM21"/>
+  <dimension ref="A1:AK21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" bestFit="1" customWidth="1"/>
@@ -2105,7 +2084,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="20" spans="1:39" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -2246,16 +2225,8 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="AK20">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-      <c r="AL20">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" spans="1:39" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -2330,10 +2301,10 @@
       <c r="X21">
         <v>1000</v>
       </c>
-      <c r="AL21">
-        <v>200</v>
-      </c>
-      <c r="AM21" t="s">
+      <c r="AJ21">
+        <v>300</v>
+      </c>
+      <c r="AK21" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>